<commit_message>
Unify database across web and mobile using canonical user ID, simplify login to username-only
</commit_message>
<xml_diff>
--- a/data/users/mghazalinurrahman939_gmail.com/MoneyTracking.xlsx
+++ b/data/users/mghazalinurrahman939_gmail.com/MoneyTracking.xlsx
@@ -29,24 +29,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <name val="Calibri"/>
+      <color rgb="000F172A"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004F46E5"/>
-        <bgColor rgb="004F46E5"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -75,10 +68,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -445,60 +444,86 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Tanggal</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Tipe</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Kategori</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Akun/Dompet</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Akun</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
         <is>
           <t>Jumlah (Rp)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Keterangan</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>ID Cicilan Terkait</t>
-        </is>
-      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ID_Cicilan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>TRX-260830215107-57E1</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Pemasukan</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Gaji</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>SeaBank</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>1400000</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Pemasukan seabank</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -513,74 +538,61 @@
   </sheetPr>
   <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ID Cicilan</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID_Cicilan</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
         <is>
           <t>Nama Cicilan</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Penyedia/Bank</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Total Pinjaman (Rp)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Cicilan/Bulan (Rp)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Total Pinjaman</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Cicilan per Bulan</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
         <is>
           <t>Tenor (Bulan)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Cicilan Ke-</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Sisa Tenor</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Sisa Hutang</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>Tgl Jatuh Tempo</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Status</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Sisa Hutang (Rp)</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Created At</t>
         </is>
       </c>
     </row>
@@ -595,76 +607,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ID Aset</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID_Aset</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
         <is>
           <t>Nama Aset</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Kategori</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Platform/Broker</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Unit/Lot</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Jumlah Unit</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
         <is>
           <t>Total Modal (Rp)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Nilai Saat Ini (Rp)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Keuntungan/PnL (Rp)</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Untung/Rugi (Rp)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
         <is>
           <t>Return (%)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Catatan</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Updated At</t>
         </is>
       </c>
     </row>
@@ -681,26 +675,21 @@
   </sheetPr>
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Kategori Pemasukan</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Kategori Pengeluaran</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Daftar Akun / Dompet</t>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Daftar Akun/Dompet</t>
         </is>
       </c>
     </row>
@@ -717,7 +706,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SeaBank</t>
+          <t>BCA</t>
         </is>
       </c>
     </row>
@@ -734,7 +723,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BCA</t>
+          <t>Mandiri</t>
         </is>
       </c>
     </row>
@@ -751,7 +740,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mandiri</t>
+          <t>BRI</t>
         </is>
       </c>
     </row>
@@ -768,7 +757,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BRI</t>
+          <t>BNI</t>
         </is>
       </c>
     </row>
@@ -785,7 +774,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BNI</t>
+          <t>Bank Jago</t>
         </is>
       </c>
     </row>
@@ -802,12 +791,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Bank Jago</t>
+          <t>Cash / Tunai</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>Kesehatan &amp; Obat</t>
@@ -815,12 +803,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cash / Tunai</t>
+          <t>GoPay</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>Hiburan &amp; Rekreasi</t>
@@ -828,12 +815,11 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GoPay</t>
+          <t>OVO</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>Sedekah &amp; Donasi</t>
@@ -841,12 +827,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>OVO</t>
+          <t>ShopeePay</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>Keluarga</t>
@@ -854,12 +839,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ShopeePay</t>
+          <t>DANA</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>Lain-lain</t>
@@ -867,7 +851,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DANA</t>
+          <t>SeaBank</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Populate August 2026 data and add manual refresh buttons in mobile app
</commit_message>
<xml_diff>
--- a/data/users/mghazalinurrahman939_gmail.com/MoneyTracking.xlsx
+++ b/data/users/mghazalinurrahman939_gmail.com/MoneyTracking.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,11 @@
       <name val="Calibri"/>
       <color rgb="000F172A"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -68,7 +73,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -77,6 +82,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -490,40 +504,39 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>TRX-260830215107-57E1</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>Pemasukan</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Gaji</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>SeaBank</t>
         </is>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" t="n">
         <v>1400000</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Pemasukan seabank</t>
-        </is>
-      </c>
-      <c r="H2" s="1" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Pemasukan SeaBank</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -536,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,6 +606,51 @@
       <c r="K1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>CICIL-260831015523-08FC</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Cicilan Konsumsi</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>SeaBank Paylater</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>1239996</v>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>103333</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Aktif</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="n">
+        <v>1136663</v>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-31 01:55</t>
         </is>
       </c>
     </row>

</xml_diff>